<commit_message>
Updated teh consolidated statement for all
</commit_message>
<xml_diff>
--- a/scratch/test_consolidated_validation.xlsx
+++ b/scratch/test_consolidated_validation.xlsx
@@ -677,6 +677,7 @@
       <c r="Q3" s="7"/>
       <c r="R3" s="7">
         <f>=SUM(C3:Q3)</f>
+        <v>186700</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -705,6 +706,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7">
         <f>=SUM(C4:Q4)</f>
+        <v>64800</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -714,51 +716,67 @@
       </c>
       <c r="C5" s="10">
         <f>=SUM(C3:C4)</f>
+        <v>115000</v>
       </c>
       <c r="D5" s="10">
         <f>=SUM(D3:D4)</f>
+        <v>8500</v>
       </c>
       <c r="E5" s="10">
         <f>=SUM(E3:E4)</f>
+        <v>15000</v>
       </c>
       <c r="F5" s="10">
         <f>=SUM(F3:F4)</f>
+        <v>54000</v>
       </c>
       <c r="G5" s="10">
         <f>=SUM(G3:G4)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="10">
         <f>=SUM(H3:H4)</f>
+        <v>0</v>
       </c>
       <c r="I5" s="10">
         <f>=SUM(I3:I4)</f>
+        <v>0</v>
       </c>
       <c r="J5" s="10">
         <f>=SUM(J3:J4)</f>
+        <v>54000</v>
       </c>
       <c r="K5" s="10">
         <f>=SUM(K3:K4)</f>
+        <v>5000</v>
       </c>
       <c r="L5" s="10">
         <f>=SUM(L3:L4)</f>
+        <v>0</v>
       </c>
       <c r="M5" s="10">
         <f>=SUM(M3:M4)</f>
+        <v>0</v>
       </c>
       <c r="N5" s="10">
         <f>=SUM(N3:N4)</f>
+        <v>0</v>
       </c>
       <c r="O5" s="10">
         <f>=SUM(O3:O4)</f>
+        <v>0</v>
       </c>
       <c r="P5" s="10">
         <f>=SUM(P3:P4)</f>
+        <v>0</v>
       </c>
       <c r="Q5" s="10">
         <f>=SUM(Q3:Q4)</f>
+        <v>0</v>
       </c>
       <c r="R5" s="10">
         <f>=SUM(R3:R4)</f>
+        <v>251500</v>
       </c>
     </row>
   </sheetData>
@@ -903,6 +921,7 @@
       <c r="O4" s="7"/>
       <c r="P4" s="7">
         <f>=SUM(C4:O4)</f>
+        <v>3500</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -929,6 +948,7 @@
       <c r="O5" s="7"/>
       <c r="P5" s="7">
         <f>=SUM(C5:O5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -938,45 +958,59 @@
       </c>
       <c r="C6" s="10">
         <f>=SUM(C4:C5)</f>
+        <v>2000</v>
       </c>
       <c r="D6" s="10">
         <f>=SUM(D4:D5)</f>
+        <v>1500</v>
       </c>
       <c r="E6" s="10">
         <f>=SUM(E4:E5)</f>
+        <v>0</v>
       </c>
       <c r="F6" s="10">
         <f>=SUM(F4:F5)</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10">
         <f>=SUM(G4:G5)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="10">
         <f>=SUM(H4:H5)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="10">
         <f>=SUM(I4:I5)</f>
+        <v>0</v>
       </c>
       <c r="J6" s="10">
         <f>=SUM(J4:J5)</f>
+        <v>0</v>
       </c>
       <c r="K6" s="10">
         <f>=SUM(K4:K5)</f>
+        <v>0</v>
       </c>
       <c r="L6" s="10">
         <f>=SUM(L4:L5)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10">
         <f>=SUM(M4:M5)</f>
+        <v>0</v>
       </c>
       <c r="N6" s="10">
         <f>=SUM(N4:N5)</f>
+        <v>0</v>
       </c>
       <c r="O6" s="10">
         <f>=SUM(O4:O5)</f>
+        <v>0</v>
       </c>
       <c r="P6" s="10">
         <f>=SUM(P4:P5)</f>
+        <v>3500</v>
       </c>
     </row>
   </sheetData>
@@ -1112,6 +1146,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7">
         <f>=SUM(C4:N4)</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1137,6 +1172,7 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7">
         <f>=SUM(C5:N5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1146,42 +1182,55 @@
       </c>
       <c r="C6" s="10">
         <f>=SUM(C4:C5)</f>
+        <v>1500</v>
       </c>
       <c r="D6" s="10">
         <f>=SUM(D4:D5)</f>
+        <v>0</v>
       </c>
       <c r="E6" s="10">
         <f>=SUM(E4:E5)</f>
+        <v>0</v>
       </c>
       <c r="F6" s="10">
         <f>=SUM(F4:F5)</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10">
         <f>=SUM(G4:G5)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="10">
         <f>=SUM(H4:H5)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="10">
         <f>=SUM(I4:I5)</f>
+        <v>0</v>
       </c>
       <c r="J6" s="10">
         <f>=SUM(J4:J5)</f>
+        <v>0</v>
       </c>
       <c r="K6" s="10">
         <f>=SUM(K4:K5)</f>
+        <v>0</v>
       </c>
       <c r="L6" s="10">
         <f>=SUM(L4:L5)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10">
         <f>=SUM(M4:M5)</f>
+        <v>0</v>
       </c>
       <c r="N6" s="10">
         <f>=SUM(N4:N5)</f>
+        <v>0</v>
       </c>
       <c r="O6" s="10">
         <f>=SUM(O4:O5)</f>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
@@ -1317,6 +1366,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7">
         <f>=SUM(C4:N4)</f>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1342,6 +1392,7 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7">
         <f>=SUM(C5:N5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1351,42 +1402,55 @@
       </c>
       <c r="C6" s="10">
         <f>=SUM(C4:C5)</f>
+        <v>200</v>
       </c>
       <c r="D6" s="10">
         <f>=SUM(D4:D5)</f>
+        <v>0</v>
       </c>
       <c r="E6" s="10">
         <f>=SUM(E4:E5)</f>
+        <v>0</v>
       </c>
       <c r="F6" s="10">
         <f>=SUM(F4:F5)</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10">
         <f>=SUM(G4:G5)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="10">
         <f>=SUM(H4:H5)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="10">
         <f>=SUM(I4:I5)</f>
+        <v>0</v>
       </c>
       <c r="J6" s="10">
         <f>=SUM(J4:J5)</f>
+        <v>0</v>
       </c>
       <c r="K6" s="10">
         <f>=SUM(K4:K5)</f>
+        <v>0</v>
       </c>
       <c r="L6" s="10">
         <f>=SUM(L4:L5)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10">
         <f>=SUM(M4:M5)</f>
+        <v>0</v>
       </c>
       <c r="N6" s="10">
         <f>=SUM(N4:N5)</f>
+        <v>0</v>
       </c>
       <c r="O6" s="10">
         <f>=SUM(O4:O5)</f>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -1522,6 +1586,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7">
         <f>=SUM(C4:N4)</f>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1547,6 +1612,7 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7">
         <f>=SUM(C5:N5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1556,42 +1622,55 @@
       </c>
       <c r="C6" s="10">
         <f>=SUM(C4:C5)</f>
+        <v>100</v>
       </c>
       <c r="D6" s="10">
         <f>=SUM(D4:D5)</f>
+        <v>0</v>
       </c>
       <c r="E6" s="10">
         <f>=SUM(E4:E5)</f>
+        <v>0</v>
       </c>
       <c r="F6" s="10">
         <f>=SUM(F4:F5)</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10">
         <f>=SUM(G4:G5)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="10">
         <f>=SUM(H4:H5)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="10">
         <f>=SUM(I4:I5)</f>
+        <v>0</v>
       </c>
       <c r="J6" s="10">
         <f>=SUM(J4:J5)</f>
+        <v>0</v>
       </c>
       <c r="K6" s="10">
         <f>=SUM(K4:K5)</f>
+        <v>0</v>
       </c>
       <c r="L6" s="10">
         <f>=SUM(L4:L5)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10">
         <f>=SUM(M4:M5)</f>
+        <v>0</v>
       </c>
       <c r="N6" s="10">
         <f>=SUM(N4:N5)</f>
+        <v>0</v>
       </c>
       <c r="O6" s="10">
         <f>=SUM(O4:O5)</f>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1727,6 +1806,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7">
         <f>=SUM(C4:N4)</f>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1752,6 +1832,7 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7">
         <f>=SUM(C5:N5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1761,42 +1842,55 @@
       </c>
       <c r="C6" s="10">
         <f>=SUM(C4:C5)</f>
+        <v>50</v>
       </c>
       <c r="D6" s="10">
         <f>=SUM(D4:D5)</f>
+        <v>0</v>
       </c>
       <c r="E6" s="10">
         <f>=SUM(E4:E5)</f>
+        <v>0</v>
       </c>
       <c r="F6" s="10">
         <f>=SUM(F4:F5)</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10">
         <f>=SUM(G4:G5)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="10">
         <f>=SUM(H4:H5)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="10">
         <f>=SUM(I4:I5)</f>
+        <v>0</v>
       </c>
       <c r="J6" s="10">
         <f>=SUM(J4:J5)</f>
+        <v>0</v>
       </c>
       <c r="K6" s="10">
         <f>=SUM(K4:K5)</f>
+        <v>0</v>
       </c>
       <c r="L6" s="10">
         <f>=SUM(L4:L5)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10">
         <f>=SUM(M4:M5)</f>
+        <v>0</v>
       </c>
       <c r="N6" s="10">
         <f>=SUM(N4:N5)</f>
+        <v>0</v>
       </c>
       <c r="O6" s="10">
         <f>=SUM(O4:O5)</f>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>